<commit_message>
subarea classificada so por codigo (palavras-chave + modelo nas ambiguas), README unico, pastas padronizadas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parte 1/DATASET_CARD.xlsx
+++ b/parte 1/DATASET_CARD.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>Versão 1.1 - atualizada em 02/10/2026 (revisão dos rótulos de subárea)</t>
+          <t>Versão 1.1 - atualizada em 02/10/2026 (classificação de subárea em duas etapas)</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="C14" s="1" t="n">
-        <v>267267</v>
+        <v>267403</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>16978</v>
+        <v>16988</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>2504</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
@@ -779,7 +779,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>O dataset possui questões de 5 subáreas da computação: Eng. Software e Programação: 720 questões (28,8%); Redes e Infraestrutura: 651 questões (26,0%); Segurança da Informação: 517 questões (20,6%); Banco de Dados e Ciência de Dados: 465 questões (18,6%); Governança e Gestão de TI: 151 questões (6,0%).</t>
+          <t>O dataset possui questões de 5 subáreas da computação: Eng. Software e Programação: 724 questões (28,9%); Redes e Infraestrutura: 674 questões (26,9%); Segurança da Informação: 505 questões (20,2%); Banco de Dados e Ciência de Dados: 464 questões (18,5%); Governança e Gestão de TI: 139 questões (5,5%). As três primeiras atendem ao mínimo de 500 questões; as duas últimas são subáreas extras.</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>Tamanho médio em tokens de cada questão (enunciado + alternativas): 106,74</t>
+          <t>Tamanho médio em tokens de cada questão (enunciado + alternativas): 106,71</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>A qualidade dos textos é a proporção de tokens alfabéticos reconhecidos em dicionário de português ou inglês (pyspellchecker); é um limite inferior, pois siglas e termos técnicos (ex.: tcp, json, kubernetes) contam como não reconhecidos. A subárea vem de um classificador de palavras-chave. Na versão 1.1, revisamos as 236 questões em que um classificador TF-IDF (validação cruzada) discordava do rótulo: 122 mudaram de subárea e 2 saíram por não serem de computação. Depois, numa amostra aleatória de 100 questões (20 por subárea), 97 estavam corretas; os 3 erros também foram corrigidos. Correções em dados/revisao_rotulos.csv; amostra em corpus/validacao_manual.json.</t>
+          <t>A qualidade dos textos é a proporção de tokens alfabéticos reconhecidos em dicionário de português ou inglês (pyspellchecker); é um limite inferior, pois siglas e termos técnicos (ex.: tcp, json, kubernetes) contam como não reconhecidos. A subárea é atribuída em duas etapas (scripts/subareas.py): pontuação por palavras-chave, com o enunciado valendo o dobro das alternativas; nas questões ambíguas (margem &lt; 4 pontos entre as duas primeiras subáreas), um TF-IDF + regressão logística treinado nas questões não ambíguas decide. Numa amostra aleatória de 100 questões conferida à mão, 95 estão na subárea correta (dados/validacao_rotulos.csv).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
subarea com k-NN (visto em aula), parte 3 refeita, parte 4 com Gemini e escala da aula
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parte 1/DATASET_CARD.xlsx
+++ b/parte 1/DATASET_CARD.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>O dataset possui questões de 5 subáreas da computação: Eng. Software e Programação: 724 questões (28,9%); Redes e Infraestrutura: 674 questões (26,9%); Segurança da Informação: 505 questões (20,2%); Banco de Dados e Ciência de Dados: 464 questões (18,5%); Governança e Gestão de TI: 139 questões (5,5%). As três primeiras atendem ao mínimo de 500 questões; as duas últimas são subáreas extras.</t>
+          <t>O dataset possui questões de 5 subáreas da computação: Eng. Software e Programação: 727 questões (29,0%); Redes e Infraestrutura: 669 questões (26,7%); Segurança da Informação: 502 questões (20,0%); Banco de Dados e Ciência de Dados: 469 questões (18,7%); Governança e Gestão de TI: 139 questões (5,5%). As três primeiras atendem ao mínimo de 500 questões; as duas últimas são subáreas extras.</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>A qualidade dos textos é a proporção de tokens alfabéticos reconhecidos em dicionário de português ou inglês (pyspellchecker); é um limite inferior, pois siglas e termos técnicos (ex.: tcp, json, kubernetes) contam como não reconhecidos. A subárea é atribuída em duas etapas (scripts/subareas.py): pontuação por palavras-chave, com o enunciado valendo o dobro das alternativas; nas questões ambíguas (margem &lt; 4 pontos entre as duas primeiras subáreas), um TF-IDF + regressão logística treinado nas questões não ambíguas decide. Numa amostra aleatória de 100 questões conferida à mão, 95 estão na subárea correta (dados/validacao_rotulos.csv).</t>
+          <t>A qualidade dos textos é a proporção de tokens alfabéticos reconhecidos em dicionário de português ou inglês (pyspellchecker); é um limite inferior, pois siglas e termos técnicos (ex.: tcp, json, kubernetes) contam como não reconhecidos. A subárea é atribuída em duas etapas (scripts/subareas.py): pontuação por palavras-chave, com o enunciado valendo o dobro das alternativas; nas questões ambíguas (margem &lt; 4 pontos entre as duas primeiras subáreas), um TF-IDF + k-NN (k=3) treinado nas questões não ambíguas decide. Numa amostra aleatória de 100 questões conferida à mão, 97 estão na subárea correta (dados/validacao_rotulos.csv).</t>
         </is>
       </c>
     </row>

</xml_diff>